<commit_message>
sprint 1, validacion, graficos de avance y control
</commit_message>
<xml_diff>
--- a/FASE 2/Evidencias Proyecto/Evidencias de documentación/Control del proyecto/control-capstone-2026-FitSearch.xlsx
+++ b/FASE 2/Evidencias Proyecto/Evidencias de documentación/Control del proyecto/control-capstone-2026-FitSearch.xlsx
@@ -1358,7 +1358,7 @@
       <c r="I12" s="43" t="n"/>
       <c r="J12" s="43" t="inlineStr">
         <is>
-          <t>Sprint 1 cerrado en horas: 11 tareas y 43 h estimadas, con 43 h reales registradas (Luis 15, Rodrigo 14, Nicolás 14). Pendiente la Sprint Review y el documento Validando Sprint 1.</t>
+          <t>Sprint 1: 11 tareas, 43 h estimadas y 43 h reales (Luis 15, Rodrigo 14, Nicolás 14). Documento Validando Sprint 1 completo con avances día a día, gráfico de avance y pila del producto actualizada; falta la aceptación del Product Owner (columna A/R) en la Sprint Review.</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       <c r="I15" s="43" t="n"/>
       <c r="J15" s="43" t="inlineStr">
         <is>
-          <t>Plantilla ya lista (Plantilla_Resumen_Reunion_Retrospectiva.docx), pendiente la primera sesión al cerrar el Sprint 1.</t>
+          <t>Plantilla lista con la identificación del Sprint 1; la completan Luis Méndez y Nicolás Silva en la reunión retrospectiva (el Product Owner no asiste).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs: aprobacion DoD de Luis, nombre FitSearch en README e instrucciones Miro actualizadas
</commit_message>
<xml_diff>
--- a/FASE 2/Evidencias Proyecto/Evidencias de documentación/Control del proyecto/control-capstone-2026-FitSearch.xlsx
+++ b/FASE 2/Evidencias Proyecto/Evidencias de documentación/Control del proyecto/control-capstone-2026-FitSearch.xlsx
@@ -669,7 +669,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="24" customHeight="1" s="23">
       <c r="A4" s="26" t="inlineStr">
         <is>
@@ -929,7 +928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A4:J17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.1484375" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="15" customWidth="1" style="22" min="1" max="2"/>
@@ -943,9 +942,6 @@
     <col width="35" customWidth="1" style="22" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="23">
       <c r="A4" s="39" t="inlineStr">
         <is>
@@ -1410,7 +1406,7 @@
       <c r="I13" s="43" t="n"/>
       <c r="J13" s="43" t="inlineStr">
         <is>
-          <t>Documento Fase 2/Definition_of_Done.docx (15 criterios por historia y 5 por sprint). Aprobado por el Product Owner el 20-09-2026; pendientes las aprobaciones de Luis Méndez y Nicolás Silva.</t>
+          <t>Documento FASE 2/Evidencias Proyecto/Evidencias de documentación/Definition_of_Done.docx (v1.5: 15 criterios por historia y 5 por sprint). Aprobado por Rodrigo Cárcamo Rojas (Product Owner) el 20-09-2026 y por Luis Méndez (Scrum Master) el 22-09-2026 mediante el pull request #1 revisado y fusionado en GitHub; pendiente la aprobación de Nicolás Silva.</t>
         </is>
       </c>
     </row>
@@ -1617,7 +1613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A4:G28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.1484375" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="22" min="1" max="1"/>
@@ -1629,9 +1625,6 @@
     <col width="35" customWidth="1" style="22" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="23">
       <c r="A4" s="39" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Registra la aprobacion de la DoD de Nicolas Silva (PR #5) en la Guia 2.4 y el control
</commit_message>
<xml_diff>
--- a/FASE 2/Evidencias Proyecto/Evidencias de documentación/Control del proyecto/control-capstone-2026-FitSearch.xlsx
+++ b/FASE 2/Evidencias Proyecto/Evidencias de documentación/Control del proyecto/control-capstone-2026-FitSearch.xlsx
@@ -1406,7 +1406,7 @@
       <c r="I13" s="43" t="n"/>
       <c r="J13" s="43" t="inlineStr">
         <is>
-          <t>Documento FASE 2/Evidencias Proyecto/Evidencias de documentación/Definition_of_Done.docx (v1.5: 15 criterios por historia y 5 por sprint). Aprobado por Rodrigo Cárcamo Rojas (Product Owner) el 20-09-2026 y por Luis Méndez (Scrum Master) el 22-09-2026 mediante el pull request #1 revisado y fusionado en GitHub; pendiente la aprobación de Nicolás Silva.</t>
+          <t>Documento FASE 2/Evidencias Proyecto/Evidencias de documentación/Definition_of_Done.docx (v1.6: 15 criterios por historia y 5 por sprint). Aprobado por Rodrigo Cárcamo Rojas (Product Owner) el 20-09-2026, por Luis Méndez (Scrum Master) el 22-09-2026 mediante el pull request #1 y por Nicolás Silva (Desarrollador) el 22-09-2026 mediante el pull request #5, ambos revisados y fusionados en GitHub.</t>
         </is>
       </c>
     </row>
@@ -1613,7 +1613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A4:G28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.1484375" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="22" min="1" max="1"/>
@@ -1625,9 +1625,6 @@
     <col width="35" customWidth="1" style="22" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="23">
       <c r="A4" s="39" t="inlineStr">
         <is>

</xml_diff>